<commit_message>
fix(workbooks): split the communication lead-lag of the IEC template
</commit_message>
<xml_diff>
--- a/workbooks/Producer_IEC.xlsx
+++ b/workbooks/Producer_IEC.xlsx
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1899" uniqueCount="745">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1927" uniqueCount="757">
   <si>
     <t>format_version</t>
   </si>
@@ -2326,6 +2326,42 @@
   </si>
   <si>
     <t>Drive train damping</t>
+  </si>
+  <si>
+    <t>tLagM</t>
+  </si>
+  <si>
+    <t>Communication lag time constant for PPC measurements in s</t>
+  </si>
+  <si>
+    <t>tLeadM</t>
+  </si>
+  <si>
+    <t>Communication lead time constant for PPC measurements in s</t>
+  </si>
+  <si>
+    <t>tLagPD</t>
+  </si>
+  <si>
+    <t>Communication lag time constant for PPC setpoints in s</t>
+  </si>
+  <si>
+    <t>tLeadPD</t>
+  </si>
+  <si>
+    <t>Communication lead time constant for PPC setpoints in s</t>
+  </si>
+  <si>
+    <t>tLagRef</t>
+  </si>
+  <si>
+    <t>Communication lag time constant for PPC references in s</t>
+  </si>
+  <si>
+    <t>tLeadRef</t>
+  </si>
+  <si>
+    <t>Communication lead time constant for PPC references in s</t>
   </si>
 </sst>
 </file>
@@ -5454,14 +5490,14 @@
         <v>388</v>
       </c>
       <c r="M5" s="97" t="s">
-        <v>432</v>
+        <v>745</v>
       </c>
       <c r="N5" s="100"/>
       <c r="O5" s="97" t="s">
         <v>336</v>
       </c>
       <c r="P5" s="103" t="s">
-        <v>433</v>
+        <v>746</v>
       </c>
       <c r="Q5" s="106" t="s">
         <v>400</v>
@@ -5495,29 +5531,29 @@
         <v>18</v>
       </c>
       <c r="I6" s="113"/>
-      <c r="K6" s="99" t="s">
-        <v>388</v>
-      </c>
-      <c r="L6" s="99" t="s">
-        <v>388</v>
-      </c>
-      <c r="M6" s="99" t="s">
-        <v>436</v>
-      </c>
-      <c r="N6" s="102"/>
-      <c r="O6" s="99" t="s">
-        <v>336</v>
-      </c>
-      <c r="P6" s="105" t="s">
-        <v>437</v>
-      </c>
-      <c r="Q6" s="110" t="s">
+      <c r="K6" s="98" t="s">
+        <v>388</v>
+      </c>
+      <c r="L6" s="98" t="s">
+        <v>388</v>
+      </c>
+      <c r="M6" s="98" t="s">
+        <v>747</v>
+      </c>
+      <c r="N6" s="101"/>
+      <c r="O6" s="98" t="s">
+        <v>336</v>
+      </c>
+      <c r="P6" s="104" t="s">
+        <v>748</v>
+      </c>
+      <c r="Q6" s="108" t="s">
         <v>400</v>
       </c>
-      <c r="R6" s="111" t="s">
+      <c r="R6" s="109" t="s">
         <v>18</v>
       </c>
-      <c r="S6" s="114"/>
+      <c r="S6" s="113"/>
     </row>
     <row r="7" spans="1:19">
       <c r="A7" s="98" t="s">
@@ -5543,6 +5579,29 @@
         <v>18</v>
       </c>
       <c r="I7" s="113"/>
+      <c r="K7" s="98" t="s">
+        <v>388</v>
+      </c>
+      <c r="L7" s="98" t="s">
+        <v>388</v>
+      </c>
+      <c r="M7" s="98" t="s">
+        <v>749</v>
+      </c>
+      <c r="N7" s="101"/>
+      <c r="O7" s="98" t="s">
+        <v>336</v>
+      </c>
+      <c r="P7" s="104" t="s">
+        <v>750</v>
+      </c>
+      <c r="Q7" s="108" t="s">
+        <v>400</v>
+      </c>
+      <c r="R7" s="109" t="s">
+        <v>18</v>
+      </c>
+      <c r="S7" s="113"/>
     </row>
     <row r="8" spans="1:19">
       <c r="A8" s="98" t="s">
@@ -5568,6 +5627,29 @@
         <v>18</v>
       </c>
       <c r="I8" s="113"/>
+      <c r="K8" s="98" t="s">
+        <v>388</v>
+      </c>
+      <c r="L8" s="98" t="s">
+        <v>388</v>
+      </c>
+      <c r="M8" s="98" t="s">
+        <v>751</v>
+      </c>
+      <c r="N8" s="101"/>
+      <c r="O8" s="98" t="s">
+        <v>336</v>
+      </c>
+      <c r="P8" s="104" t="s">
+        <v>752</v>
+      </c>
+      <c r="Q8" s="108" t="s">
+        <v>400</v>
+      </c>
+      <c r="R8" s="109" t="s">
+        <v>18</v>
+      </c>
+      <c r="S8" s="113"/>
     </row>
     <row r="9" spans="1:19">
       <c r="A9" s="98" t="s">
@@ -5593,6 +5675,29 @@
         <v>18</v>
       </c>
       <c r="I9" s="113"/>
+      <c r="K9" s="98" t="s">
+        <v>388</v>
+      </c>
+      <c r="L9" s="98" t="s">
+        <v>388</v>
+      </c>
+      <c r="M9" s="98" t="s">
+        <v>753</v>
+      </c>
+      <c r="N9" s="101"/>
+      <c r="O9" s="98" t="s">
+        <v>336</v>
+      </c>
+      <c r="P9" s="104" t="s">
+        <v>754</v>
+      </c>
+      <c r="Q9" s="108" t="s">
+        <v>400</v>
+      </c>
+      <c r="R9" s="109" t="s">
+        <v>18</v>
+      </c>
+      <c r="S9" s="113"/>
     </row>
     <row r="10" spans="1:19">
       <c r="A10" s="99" t="s">
@@ -5618,6 +5723,29 @@
         <v>18</v>
       </c>
       <c r="I10" s="114"/>
+      <c r="K10" s="99" t="s">
+        <v>388</v>
+      </c>
+      <c r="L10" s="99" t="s">
+        <v>388</v>
+      </c>
+      <c r="M10" s="99" t="s">
+        <v>755</v>
+      </c>
+      <c r="N10" s="102"/>
+      <c r="O10" s="99" t="s">
+        <v>336</v>
+      </c>
+      <c r="P10" s="105" t="s">
+        <v>756</v>
+      </c>
+      <c r="Q10" s="110" t="s">
+        <v>400</v>
+      </c>
+      <c r="R10" s="111" t="s">
+        <v>18</v>
+      </c>
+      <c r="S10" s="114"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>